<commit_message>
Rewrite Sugar News summary for 2026-08-17
</commit_message>
<xml_diff>
--- a/reports/2026/08/Sugar News 2026-08-17.xlsx
+++ b/reports/2026/08/Sugar News 2026-08-17.xlsx
@@ -505,7 +505,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="134" customHeight="1" s="2">
+    <row r="2" ht="180" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -513,16 +513,16 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>印度糖厂发布或调整糖厂运行和压榨安排，相关数值为97 crore、Rs 97。印度糖厂若增加开工或压榨，会加快当季食糖产出；若停产或延后开榨，则阶段性供应收紧。来源：ChiniMandi（https://www.chinimandi.com/bihar-approves-rs-97-crore-revival-of-sakri-sugar-mill-after-29-years/）。影响：利空糖价</t>
+          <t>印度比哈尔邦政府批准重建马杜巴尼县Sakri糖厂，并同步推进达尔班加县Raiyam糖厂重建；Sakri项目预计投资约9.7亿卢比，包含食糖和乙醇生产设施，原厂1933年建成、1997年停产。重建将为Madhubani及周边甘蔗提供本地收购和压榨渠道，可能带动甘蔗种植面积恢复并提高印度未来食糖和乙醇加工能力，增加中长期供应预期。项目仍处重建准备期，对短期现货供应影响有限。来源：ChiniMandi（https://www.chinimandi.com/bihar-approves-rs-97-crore-revival-of-sakri-sugar-mill-after-29-years/）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>利空：糖厂运行、压榨能力或原料供应改善会提高食糖生产节奏，增加阶段性供应。</t>
+          <t>利空：糖厂重建和甘蔗面积恢复会提高未来压榨与食糖产出能力，增加印度中长期供应；但项目仍在重建阶段，短期影响有限。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="160.4" customHeight="1" s="2">
+    <row r="3" ht="180" customHeight="1" s="2">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -530,16 +530,16 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>印度糖业相关机构公布库存数据，库存增加7%。库存增加会提高现货供应缓冲，压制补库需求和糖价。来源：The Economic Times（https://m.economictimes.com/markets/stocks/news/sugar-stocks-balrampur-chini-triveni-engineering-dhampur-sugar-and-others-rally-up-to-7-heres-why/articleshow/133288064.cms）。影响：利空糖价</t>
+          <t>印度糖业股在8月17日最高上涨约7%，《经济时报》称推动因素包括国际原糖升至16.6美分/磅、白糖触及15个月高位，孟买现货糖价一个月上涨近10%至约5000-5090卢比/公担。价格上涨叠加印度降雨不足和节庆需求预期，反映印度现货供应偏紧和需求前置补库，对国内糖价形成支撑。来源：The Economic Times（https://m.economictimes.com/markets/stocks/news/sugar-stocks-balrampur-chini-triveni-engineering-dhampur-sugar-and-others-rally-up-to-7-heres-why/articleshow/133288064.cms）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>利空：库存增加会提高现货供应缓冲，压制补库需求和糖价。</t>
+          <t>偏多糖价：现货糖价大幅上涨、雨量偏少和节庆需求预期共同指向印度阶段性供需偏紧，支撑糖价。</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="135.65" customHeight="1" s="2">
+    <row r="4" ht="180" customHeight="1" s="2">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -547,46 +547,46 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>印度糖业相关机构下调食糖贸易、进口、出口或配额政策，相关数值为1 billion、$1。进口、出口、关税或配额变化会改变国内外可用糖源和贸易流向。来源：ChiniMandi（https://www.chinimandi.com/nigerian-sugar-industry-gets-1-billion-investment-push-to-cut-import-dependence/）。影响：利空糖价</t>
+          <t>印度首席经济顾问V. Anantha Nageswaran与经济事务部顾问Akash Poojari建议为老旧两轮车恢复E10汽油，并在把乙醇掺混率从已实现的20%继续推向E27、E30前评估粮食、土地和用水成本。若政策放慢20%以上掺混提升，糖厂新增乙醇需求将减少，甘蔗汁、糖浆或B重糖蜜转入乙醇的压力下降，更多可结晶糖源可用于制糖，利空糖价。该意见尚非最终政策，影响主要体现在后续乙醇掺混政策预期。来源：ChiniMandi（https://www.chinimandi.com/cea-urges-caution-on-higher-ethanol-blending-backs-e10-option-for-older-two-wheelers/）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>利空：进口政策放宽或进口量增加会补充国内可用糖源，对本地糖价形成压力。</t>
+          <t>利空：放缓高于E20的乙醇掺混会减少糖基乙醇增量需求，降低对甘蔗汁、糖浆和B重糖蜜的分流，使更多蔗糖原料可用于制糖。</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="151.05" customHeight="1" s="2">
+    <row r="5" ht="180" customHeight="1" s="2">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>泰国</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>印度糖业相关机构公布乙醇掺混或燃料政策，相关数值为E10。若新增乙醇需求由B重糖蜜、糖浆或甘蔗汁满足，糖厂会把这些可发酵糖源送入乙醇装置；其中B重糖蜜、糖浆和甘蔗汁会减少可结晶成白糖的蔗糖量。来源：ChiniMandi（https://www.chinimandi.com/cea-urges-caution-on-higher-ethanol-blending-backs-e10-option-for-older-two-wheelers/）。影响：利多糖价</t>
+          <t>Open-Meteo预报显示（2026-08-18至2026-08-24），泰国东北部（呵叻、孔敬、乌隆他尼、猜也蓬）；北部（那空沙旺、甘烹碧、素可泰、彭世洛）；中部及西部（北碧、华富里、素攀武里、猜纳）；东部（沙缴、春武里）等主要甘蔗产区存在降雨预报，实际可用预报期为7日，累计预测降雨较高的监测点包括加拉信约121.7mm、乌隆他尼约118.3mm、黎府约117.4mm。当前处于甘蔗生长阶段，降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：Open-Meteo（https://api.open-meteo.com/v1/forecast）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>利多：若新增乙醇需求由B重糖蜜、糖浆或甘蔗汁满足，糖厂会把这些可发酵糖源送入乙醇装置；其中B重糖蜜、糖浆和甘蔗汁会减少可结晶成白糖的蔗糖量，从而减少食糖供应预期并支撑糖价。</t>
+          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="180" customHeight="1" s="2">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>泰国</t>
+          <t>尼日利亚</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Open-Meteo预报显示（2026-08-18至2026-08-24），泰国东北部（呵叻、孔敬、乌隆他尼、猜也蓬）；北部（那空沙旺、甘烹碧、素可泰、彭世洛）；中部及西部（北碧、华富里、素攀武里、猜纳）；东部（沙缴、春武里）等主要甘蔗产区存在降雨预报，实际可用预报期为7日，累计预测降雨较高的监测点包括加拉信约121.7mm、乌隆他尼约118.3mm、黎府约117.4mm。当前处于甘蔗生长阶段，降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：Open-Meteo（https://api.open-meteo.com/v1/forecast）。影响：利空糖价</t>
+          <t>尼日利亚国家糖业发展委员会（NSDC）披露超过10亿美元投资计划，用于提升本土食糖产量并降低进口依赖；尼日利亚年食糖消费约180万吨，目前多数依靠进口，计划包括10亿美元EPC+融资合作和100亿奈拉糖业项目加速基金。NSMP 2.0把本土产量目标定在约200万吨/年，若项目落地将减少尼日利亚对进口糖的需求，削弱国际贸易流入需求，偏利空国际糖价。项目处于投资和执行推进阶段，对短期现货供应影响有限。来源：ChiniMandi（https://www.chinimandi.com/nigerian-sugar-industry-gets-1-billion-investment-push-to-cut-import-dependence/）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
+          <t>利空：尼日利亚本土产量目标若落地，将减少其进口糖需求并削弱国际贸易流入需求；但项目仍处推进阶段，短期影响有限。</t>
         </is>
       </c>
     </row>

</xml_diff>